<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.001-05 Victorina dit stop
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.001-05.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.001-05.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le câlin du salon</t>
+          <t>Victorina dit stop</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>salon, table, lampe, pile de livres, livre d'images, pages, carton, rond de lumière</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amir, Chouchou, maman</t>
+          <t>Victorina, Nino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir joue au salon avec Chouchou. Le câlin est trop fort. Amir dit stop, s'éloigne, rejoint maman près du radiateur.</t>
+          <t>Un rond de lumière dort sur la table. Sur le dos du livre, un éclat de livre luit. Victorina veut jouer, maintenant. Nino serre trop. Poitrine coincée, sourire parti. Papa s'accroupit. Stop. Elle recule. Merci vécu. Le livre glisse. Nino serre pour aider. Stop, recule. Un éclat de livre tient sur le dos.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le radiateur fait tic tic. Des chaussettes bleues sèchent dessus. La fenêtre est un peu embuée. Ça sent le savon chaud. Maman plie une serviette. Elle est encore tiède, Amir. Tu as senti le savon ? Oui, maman. Un bateau en bois attend. Il est sur l'étagère. Le tapis est doux et épais. En ce moment, Amir joue. Chouchou joue avec lui. Ils sont au salon. Chouchou fait un gros câlin. Le câlin est trop fort. Amir est gêné. C'est trop près. Sa poitrine est coincée. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Amir recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le canapé. Maman est l'adulte sur le canapé. Maman, c'était trop. Tu as reculé. Tu as dit stop. Bravo, Amir. Tu es venu me le dire. Tu veux ta main dans ma main ? Oui, maman. Amir pose sa main. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Chouchou prend le bateau en bois. Il le fait glisser loin. Le salon redevient calme. Amir regarde les chaussettes bleues. Elles bougent un tout petit peu. Elles sèchent, tu vois ? Oui. Elles bougent. La fenêtre a encore de la buée. Amir trace un petit trait. Le trait disparaît. Tu es bien près de moi. On reste encore un peu ? Oui, maman.</t>
+          <t>Un rond de lumière dort sur la table. Il est chaud, papa. Tu le vois, le rond ? Oui, papa. Ça sent le papier, un peu sec. Tu le sens, le papier ? Oui, maman. Une page se lève un peu. Elle bouge, maman. Le livre est là, sous la lampe. Je le vois. Papa tapote le dos du livre. Toc, toc, sur le carton. Tu entends le carton, Victorina ? Oui, il sonne. Maman pose la main près de la lampe. La lampe est tiède, un peu ronde. Sur le dos, un éclat de livre luit. Il luit, papa. Tu le vois, sur le dos ? Oui, un petit point. La lumière le touche. Un rayon glisse le long des livres. Victorina connaît cette table. Le point est nouveau. Tu t'assois près du livre ? Un peu. Un coin de page se plie. Il est plié. La page a un pli, tu vois ? Oui, papa. Le livre d'images attend sous la lampe. En ce moment, Victorina le prend. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. Le carton est lisse, un peu tiède. Tu tournes une page ? Oui, maman. Nino arrive dans le salon. Il serre trop. Il saute près de la table. Le livre ! Tu viens, Nino ? Oui. Victorina ouvre le livre trop vite. Nino passe les bras autour. Le câlin est trop fort. Le livre reste fermé. Oh. Je te tiens. Le sourire de Victorina disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules montent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Victorina ? Oui, papa. Tes bras sont coincés, Victorina ? Un peu, maman. C'est trop. Stop. Victorina recule d'un pas. L'éclat de livre tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le radiateur fait tic tic. Des chaussettes bleues sèchent dessus. La fenêtre est un peu embuée. Ça sent le savon chaud. Maman plie une serviette. Elle est encore tiède, Amir. Tu as senti le savon ? Oui, maman. Un bateau en bois attend. Il est sur l'étagère. Le tapis est doux et épais. En ce moment, Amir joue. Chouchou joue avec lui. Ils sont au salon. Chouchou fait un gros câlin. Le câlin est trop fort. Amir est gêné. C'est trop près. Sa poitrine est coincée. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Amir recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le canapé. Maman est l'adulte sur le canapé. Maman, c'était trop. Tu as reculé. Tu as dit stop. Bravo, Amir. Tu es venu me le dire. Tu veux ta main dans ma main ? Oui, maman. Amir pose sa main. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Chouchou prend le bateau en bois. Il le fait glisser loin. Le salon redevient calme. Amir regarde les chaussettes bleues. Elles bougent un tout petit peu. Elles sèchent, tu vois ? Oui. Elles bougent. La fenêtre a encore de la buée. Amir trace un petit trait. Le trait disparaît. Tu es bien près de moi. On reste encore un peu ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rond de lumière dort sur la table. Il est chaud, papa. Tu le vois, le rond ? Oui, papa. Ça sent le papier, un peu sec. Tu le sens, le papier ? Oui, maman. Une page se lève un peu. Elle bouge, maman. Le livre est là, sous la lampe. Je le vois. Papa tapote le dos du livre. Toc, toc, sur le carton. Tu entends le carton, Victorina ? Oui, il sonne. Maman pose la main près de la lampe. La lampe est tiède, un peu ronde. Sur le dos, un &lt;emphasis level="moderate"&gt;éclat de livre&lt;/emphasis&gt; luit. Il luit, papa. Tu le vois, sur le dos ? Oui, un petit point. La lumière le touche. Un rayon glisse le long des livres. Victorina connaît cette table. Le point est nouveau. Tu t'assois près du livre ? Un peu. Un coin de page se plie. Il est plié. La page a un pli, tu vois ? Oui, papa. Le livre d'images attend sous la lampe. En ce moment, Victorina le prend. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. Le carton est lisse, un peu tiède. Tu tournes une page ? Oui, maman. Nino arrive dans le salon. Il serre trop. Il saute près de la table. Le livre ! Tu viens, Nino ? Oui. Victorina ouvre le livre trop vite. Nino passe les bras autour. Le câlin est trop fort. Le livre reste fermé. Oh. Je te tiens. Le sourire de Victorina disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules montent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Victorina ? Oui, papa. Tes bras sont coincés, Victorina ? Un peu, maman. C'est trop. Stop. Victorina recule d'un pas. L'éclat de livre tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Fleur joue au salon. Un camarade la serre. Fleur sent sa poitrine. C'est trop. Fleur dit : &lt;emphasis&gt;stop&lt;/emphasis&gt;. Elle recule d'un pas. Elle peut s'éloigner. Elle s'éloigne vers le canapé. Maman est l'adulte. Fleur va vers maman. Elle dit : c'était trop. Maman l'écoute. Fleur pose sa main. Elle souffle. Dire stop, c'est permis. On s'éloigne. On va vers un adulte.&lt;/slow&gt; [pause]</t>
+          <t>Un rond de lumière dort sur la table. Il est chaud, papa. Tu le vois, le rond ? Oui, papa. Ça sent le papier, un peu sec. Tu le sens, le papier ? Oui, maman. Une page se lève un peu. Elle bouge, maman. Le livre est là, sous la lampe. Je le vois. Papa tapote le dos du livre. Toc, toc, sur le carton. Tu entends le carton, Victorina ? Oui, il sonne. Maman pose la main près de la lampe. La lampe est tiède, un peu ronde. Sur le dos, un &lt;emphasis&gt;éclat de livre&lt;/emphasis&gt; luit. Il luit, papa. Tu le vois, sur le dos ? Oui, un petit point. La lumière le touche. Un rayon glisse le long des livres. Victorina connaît cette table. Le point est nouveau. Tu t'assois près du livre ? Un peu. Un coin de page se plie. Il est plié. La page a un pli, tu vois ? Oui, papa. Le livre d'images attend sous la lampe. En ce moment, Victorina le prend. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. Le carton est lisse, un peu tiède. Tu tournes une page ? Oui, maman. Nino arrive dans le salon. Il serre trop. Il saute près de la table. Le livre ! Tu viens, Nino ? Oui. Victorina ouvre le livre trop vite. Nino passe les bras autour. Le câlin est trop fort. Le livre reste fermé. Oh. Je te tiens. Le sourire de Victorina disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules montent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Victorina ? Oui, papa. Tes bras sont coincés, Victorina ? Un peu, maman. C'est trop. Stop. Victorina recule d'un pas. L'éclat de livre tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>éclat de livre</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,64 +1324,79 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis gêne; intensite=2; destinataire=enfant; sous_texte=elle_veut_jouer_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le radiateur fait tic tic.
-narrateur|Des chaussettes bleues sèchent dessus.
-narrateur|La fenêtre est un peu embuée.
-narrateur|Ça sent le savon chaud.
-narrateur|Maman plie une serviette.
-maman|Elle est encore tiède, Amir.
-maman|Tu as senti le savon ?
-enfant-m|Oui, maman.
-narrateur|Un bateau en bois attend.
-narrateur|Il est sur l'étagère.
-narrateur|Le tapis est doux et épais.
-narrateur|En ce moment, Amir joue.
-narrateur|Chouchou joue avec lui.
-narrateur|Ils sont au salon.
-narrateur|Chouchou fait un gros câlin.
+          <t>narrateur|Un rond de lumière dort sur la table.
+enfant-f|Il est chaud, papa.
+papa|Tu le vois, le rond ?
+enfant-f|Oui, papa.
+narrateur|Ça sent le papier, un peu sec.
+maman|Tu le sens, le papier ?
+enfant-f|Oui, maman.
+narrateur|Une page se lève un peu.
+enfant-f|Elle bouge, maman.
+maman|Le livre est là, sous la lampe.
+enfant-f|Je le vois.
+narrateur|Papa tapote le dos du livre.
+narrateur|Toc, toc, sur le carton.
+papa|Tu entends le carton, Victorina ?
+enfant-f|Oui, il sonne.
+narrateur|Maman pose la main près de la lampe.
+narrateur|La lampe est tiède, un peu ronde.
+narrateur|Sur le dos, un éclat de livre luit.
+enfant-f|Il luit, papa.
+papa|Tu le vois, sur le dos ?
+enfant-f|Oui, un petit point.
+maman|La lumière le touche.
+narrateur|Un rayon glisse le long des livres.
+narrateur|Victorina connaît cette table.
+enfant-f|Le point est nouveau.
+maman|Tu t'assois près du livre ?
+enfant-f|Un peu.
+narrateur|Un coin de page se plie.
+enfant-f|Il est plié.
+papa|La page a un pli, tu vois ?
+enfant-f|Oui, papa.
+narrateur|Le livre d'images attend sous la lampe.
+narrateur|En ce moment, Victorina le prend.
+enfant-f|Je veux jouer, maintenant !
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|Le carton est lisse, un peu tiède.
+maman|Tu tournes une page ?
+enfant-f|Oui, maman.
+narrateur|Nino arrive dans le salon.
+narrateur|Il serre trop.
+narrateur|Il saute près de la table.
+copain|Le livre !
+enfant-f|Tu viens, Nino ?
+copain|Oui.
+narrateur|Victorina ouvre le livre trop vite.
+narrateur|Nino passe les bras autour.
 narrateur|Le câlin est trop fort.
-narrateur|Amir est gêné.
-narrateur|C'est trop près.
-narrateur|Sa poitrine est coincée.
-narrateur|Ses épaules montent.
-enfant-m|Je n'aime pas.
-enfant-m|C'est trop.
-enfant-m|Stop.
-narrateur|Amir recule d'un pas.
-narrateur|Il peut s'éloigner.
-narrateur|Il s'éloigne vers le canapé.
-narrateur|Maman est l'adulte sur le canapé.
-enfant-m|Maman, c'était trop.
-maman|Tu as reculé.
-maman|Tu as dit stop.
-maman|Bravo, Amir.
-maman|Tu es venu me le dire.
-maman|Tu veux ta main dans ma main ?
-enfant-m|Oui, maman.
-narrateur|Amir pose sa main.
-narrateur|Il souffle.
-narrateur|Ses épaules descendent.
-maman|Dire stop, c'est permis.
-maman|On s'éloigne.
-maman|On va vers un adulte.
-narrateur|Chouchou prend le bateau en bois.
-narrateur|Il le fait glisser loin.
-narrateur|Le salon redevient calme.
-narrateur|Amir regarde les chaussettes bleues.
-narrateur|Elles bougent un tout petit peu.
-maman|Elles sèchent, tu vois ?
-enfant-m|Oui. Elles bougent.
-narrateur|La fenêtre a encore de la buée.
-narrateur|Amir trace un petit trait.
-narrateur|Le trait disparaît.
-maman|Tu es bien près de moi.
-maman|On reste encore un peu ?
-enfant-m|Oui, maman.</t>
+narrateur|Le livre reste fermé.
+enfant-f|Oh.
+copain|Je te tiens.
+narrateur|Le sourire de Victorina disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules montent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Nino, Victorina ?
+enfant-f|Oui, papa.
+maman|Tes bras sont coincés, Victorina ?
+enfant-f|Un peu, maman.
+enfant-f|C'est trop.
+enfant-f|Stop.
+narrateur|Victorina recule d'un pas.
+narrateur|L'éclat de livre tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1413,17 +1428,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Amir. Que dit-il ?</t>
+          <t>C'est trop pour Victorina. Que dit-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Amir. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;C'est &lt;emphasis level="moderate"&gt;trop&lt;/emphasis&gt; pour Victorina. Que dit-elle ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est trop pour Fleur. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;C'est &lt;emphasis&gt;trop&lt;/emphasis&gt; pour Victorina. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1486,7 +1501,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1497,7 +1512,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1512,34 +1527,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>trop</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1554,7 +1573,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1564,12 +1583,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=c_est_trop_que_dit_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|C'est trop pour Amir. Que dit-il ?</t>
+          <t>narrateur|C'est trop pour Victorina.
+narrateur|Que dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1596,17 +1616,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir a dit stop. Il a pu s'éloigner. Il a rejoint maman, l'adulte. Tu as dit stop. Bravo. Tu restes près de moi ? Oui. La serviette est encore tiède. Le radiateur fait tic tic.</t>
+          <t>Victorina garde un pas d'air. Le livre, là. Elle pose le livre sur la table. Je m'approche. Nino se penche trop. Un peu loin. Nino recule d'un pas, lui aussi. D'accord. Tu veux le livre avec Nino ? Oui, chacun un bord. Nino ne dit rien, d'abord. Je tiens ma page. Moi aussi. Merci, Victorina. Papa a vu les deux, près de la lampe. Le papier colle un peu, sous les doigts. Il est sec. Ils essuient la page du plat de la main. Nino tient sa page, plus loin. Elle tourne ! Oui. Tu la vois, la bête ? Oui, papa. Au milieu, Nino ? J'y vais. Victorina pousse la page, sans se presser. Nino suit l'image des yeux. La page danse une fois. Un. Deux. Le ventre de Victorina se desserre. Les épaules descendent un peu. On reste près de la table ? Oui. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir a dit stop. Il a pu s'éloigner. Il a rejoint maman, l'adulte. Tu as dit stop. Bravo. Tu restes près de moi ? Oui. La serviette est encore tiède. Le radiateur fait tic tic.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina garde un pas d'air. Le &lt;emphasis level="moderate"&gt;livre&lt;/emphasis&gt;, là. Elle pose le livre sur la table. Je m'approche. Nino se penche trop. Un peu loin. Nino recule d'un pas, lui aussi. D'accord. Tu veux le livre avec Nino ? Oui, chacun un bord. Nino ne dit rien, d'abord. Je tiens ma page. Moi aussi. Merci, Victorina. Papa a vu les deux, près de la lampe. Le papier colle un peu, sous les doigts. Il est sec. Ils essuient la page du plat de la main. Nino tient sa page, plus loin. Elle tourne ! Oui. Tu la vois, la bête ? Oui, papa. Au milieu, Nino ? J'y vais. Victorina pousse la page, sans se presser. Nino suit l'image des yeux. La page danse une fois. Un. Deux. Le ventre de Victorina se desserre. Les épaules descendent un peu. On reste près de la table ? Oui. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Fleur a dit &lt;emphasis&gt;stop&lt;/emphasis&gt;. Elle a pu s'éloigner. Elle rejoint maman, l'adulte.&lt;/slow&gt; [pause]</t>
+          <t>Victorina garde un pas d'air. Le &lt;emphasis&gt;livre&lt;/emphasis&gt;, là. Elle pose le livre sur la table. Je m'approche. Nino se penche trop. Un peu loin. Nino recule d'un pas, lui aussi. D'accord. Tu veux le livre avec Nino ? Oui, chacun un bord. Nino ne dit rien, d'abord. Je tiens ma page. Moi aussi. Merci, Victorina. Papa a vu les deux, près de la lampe. Le papier colle un peu, sous les doigts. Il est sec. Ils essuient la page du plat de la main. Nino tient sa page, plus loin. Elle tourne ! Oui. Tu la vois, la bête ? Oui, papa. Au milieu, Nino ? J'y vais. Victorina pousse la page, sans se presser. Nino suit l'image des yeux. La page danse une fois. Un. Deux. Le ventre de Victorina se desserre. Les épaules descendent un peu. On reste près de la table ? Oui. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1653,18 +1673,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1687,30 +1707,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>livre</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1719,10 +1739,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1731,24 +1751,51 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_garde_un_pas_ils_tiennent; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir a dit stop.
-narrateur|Il a pu s'éloigner.
-narrateur|Il a rejoint maman, l'adulte.
-maman|Tu as dit stop.
-maman|Bravo.
-maman|Tu restes près de moi ?
-enfant-m|Oui.
-narrateur|La serviette est encore tiède.
-narrateur|Le radiateur fait tic tic.</t>
+          <t>narrateur|Victorina garde un pas d'air.
+enfant-f|Le livre, là.
+narrateur|Elle pose le livre sur la table.
+copain|Je m'approche.
+narrateur|Nino se penche trop.
+enfant-f|Un peu loin.
+narrateur|Nino recule d'un pas, lui aussi.
+copain|D'accord.
+papa|Tu veux le livre avec Nino ?
+enfant-f|Oui, chacun un bord.
+narrateur|Nino ne dit rien, d'abord.
+copain|Je tiens ma page.
+enfant-f|Moi aussi.
+papa|Merci, Victorina.
+narrateur|Papa a vu les deux, près de la lampe.
+maman|Le papier colle un peu, sous les doigts.
+enfant-f|Il est sec.
+narrateur|Ils essuient la page du plat de la main.
+narrateur|Nino tient sa page, plus loin.
+enfant-f|Elle tourne !
+copain|Oui.
+papa|Tu la vois, la bête ?
+enfant-f|Oui, papa.
+maman|Au milieu, Nino ?
+copain|J'y vais.
+narrateur|Victorina pousse la page, sans se presser.
+narrateur|Nino suit l'image des yeux.
+narrateur|La page danse une fois.
+copain|Un.
+enfant-f|Deux.
+narrateur|Le ventre de Victorina se desserre.
+narrateur|Les épaules descendent un peu.
+papa|On reste près de la table ?
+enfant-f|Oui.
+maman|Tes mains sont au chaud ?
+enfant-f|Un peu, maman.</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1822,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Amir reste près du canapé. Maman lui parle tout bas. Ta poitrine était coincée. Tu as écouté. Tu es plus calme, maintenant ? Oui, maman. Le bateau en bois attend sur le tapis. Amir souffle encore une fois. Chouchou pousse le bateau tout seul. Le bateau va loin. Toi, tu restes ici. Près de moi.</t>
+          <t>Maman pousse la pile vers le bord. La pile est un peu haute. Le livre, maintenant ! Nino avance trop, tout de suite. Il saute vers le livre. À moi ! Le livre glisse vers le bord. Il part ! Victorina avance les mains, trop vite. Nino la serre pour l'aider. Les bras ferment trop. Oh. Victorina refuse d'avancer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le livre, un instant. Elle écoute le carton de la table. Sur le dos, un éclat de livre luit. Là, sur le dos. Stop. Victorina recule d'un pas. Tu tends les doigts, Nino ? Nino ne dit rien. Il souffle, puis tend les doigts. Oui. On arrête le livre ? Oui, papa. Le dos sent le carton tiède. Le livre est là, un peu au bord. Victorina le pose près de Nino. Nino le rend, sans serrer. Frou. Frou. La page est bien ouverte ? Oui, papa. Le papier est sec, Nino ? Un peu. Ils se passent la page, près d'eux. La table est lisse, sous les genoux. C'est plus facile. La lampe est calme ? Oui, papa. Un rayon passe sur le dos. Il allume le point.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Amir reste près du canapé. Maman lui parle tout bas. Ta poitrine était coincée. Tu as écouté. Tu es plus calme, maintenant ? Oui, maman. Le bateau en bois attend sur le tapis. Amir souffle encore une fois. Chouchou pousse le bateau tout seul. Le bateau va loin. Toi, tu restes ici. Près de moi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pousse la pile vers le bord. La pile est un peu haute. Le livre, maintenant ! Nino avance trop, tout de suite. Il saute vers le livre. À moi ! Le livre glisse vers le bord. Il part ! Victorina avance les mains, trop vite. Nino la serre pour l'aider. Les bras ferment trop. Oh. Victorina refuse d'avancer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le livre, un instant. Elle écoute le carton de la table. Sur le dos, un &lt;emphasis level="moderate"&gt;éclat de livre&lt;/emphasis&gt; luit. Là, sur le dos. Stop. Victorina recule d'un pas. Tu tends les doigts, Nino ? Nino ne dit rien. Il souffle, puis tend les doigts. Oui. On arrête le livre ? Oui, papa. Le dos sent le carton tiède. Le livre est là, un peu au bord. Victorina le pose près de Nino. Nino le rend, sans serrer. Frou. Frou. La page est bien ouverte ? Oui, papa. Le papier est sec, Nino ? Un peu. Ils se passent la page, près d'eux. La table est lisse, sous les genoux. C'est plus facile. La lampe est calme ? Oui, papa. Un rayon passe sur le dos. Il allume le point.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Fleur reste près du canapé. Maman lui parle tout bas.&lt;/slow&gt; [pause]</t>
+          <t>Maman pousse la pile vers le bord. La pile est un peu haute. Le livre, maintenant ! Nino avance trop, tout de suite. Il saute vers le livre. À moi ! Le livre glisse vers le bord. Il part ! Victorina avance les mains, trop vite. Nino la serre pour l'aider. Les bras ferment trop. Oh. Victorina refuse d'avancer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le livre, un instant. Elle écoute le carton de la table. Sur le dos, un &lt;emphasis&gt;éclat de livre&lt;/emphasis&gt; luit. Là, sur le dos. Stop. Victorina recule d'un pas. Tu tends les doigts, Nino ? Nino ne dit rien. Il souffle, puis tend les doigts. Oui. On arrête le livre ? Oui, papa. Le dos sent le carton tiède. Le livre est là, un peu au bord. Victorina le pose près de Nino. Nino le rend, sans serrer. Frou. Frou. La page est bien ouverte ? Oui, papa. Le papier est sec, Nino ? Un peu. Ils se passent la page, près d'eux. La table est lisse, sous les genoux. C'est plus facile. La lampe est calme ? Oui, papa. Un rayon passe sur le dos. Il allume le point. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1832,18 +1879,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1864,28 +1911,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de livre</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1894,10 +1945,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1906,23 +1957,59 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=le_livre_glisse_nino_serre_pour_aider; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Amir reste près du canapé.
-narrateur|Maman lui parle tout bas.
-maman|Ta poitrine était coincée.
-maman|Tu as écouté.
-maman|Tu es plus calme, maintenant ?
-enfant-m|Oui, maman.
-narrateur|Le bateau en bois attend sur le tapis.
-narrateur|Amir souffle encore une fois.
-narrateur|Chouchou pousse le bateau tout seul.
-narrateur|Le bateau va loin.
-maman|Toi, tu restes ici.
-maman|Près de moi.</t>
+          <t>narrateur|Maman pousse la pile vers le bord.
+narrateur|La pile est un peu haute.
+enfant-f|Le livre, maintenant !
+narrateur|Nino avance trop, tout de suite.
+narrateur|Il saute vers le livre.
+copain|À moi !
+narrateur|Le livre glisse vers le bord.
+enfant-f|Il part !
+narrateur|Victorina avance les mains, trop vite.
+narrateur|Nino la serre pour l'aider.
+narrateur|Les bras ferment trop.
+enfant-f|Oh.
+narrateur|Victorina refuse d'avancer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le livre, un instant.
+narrateur|Elle écoute le carton de la table.
+narrateur|Sur le dos, un éclat de livre luit.
+enfant-f|Là, sur le dos.
+enfant-f|Stop.
+narrateur|Victorina recule d'un pas.
+enfant-f|Tu tends les doigts, Nino ?
+narrateur|Nino ne dit rien.
+narrateur|Il souffle, puis tend les doigts.
+copain|Oui.
+papa|On arrête le livre ?
+enfant-f|Oui, papa.
+narrateur|Le dos sent le carton tiède.
+narrateur|Le livre est là, un peu au bord.
+narrateur|Victorina le pose près de Nino.
+narrateur|Nino le rend, sans serrer.
+enfant-f|Frou.
+copain|Frou.
+papa|La page est bien ouverte ?
+enfant-f|Oui, papa.
+maman|Le papier est sec, Nino ?
+copain|Un peu.
+narrateur|Ils se passent la page, près d'eux.
+narrateur|La table est lisse, sous les genoux.
+enfant-f|C'est plus facile.
+papa|La lampe est calme ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le dos.
+enfant-f|Il allume le point.</t>
         </is>
       </c>
     </row>
@@ -1949,17 +2036,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloigné. Je suis allé vers maman. Bravo.</t>
+          <t>Ils restent près de la lampe. Maman lisse un coin de page. Le livre a glissé, papa. Tu l'as vu, toi ? Oui, près de la table. On est bien, ici. Victorina tapote le dos du doigt. Il a une trace de doigt. Tu la vois, la trace ? Oui, maman. Le livre est resté, Victorina. Oui, avec Nino. Le livre est resté. Ça sent le papier, un peu tiède. Et le carton, maman. Oui, dans l'air. Le livre reste sous la lampe. Un éclat de livre tient sur le dos.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloigné. Je suis allé vers maman. Bravo.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la lampe. Maman lisse un coin de page. Le livre a glissé, papa. Tu l'as vu, toi ? Oui, près de la table. On est bien, ici. Victorina tapote le dos du doigt. Il a une trace de doigt. Tu la vois, la trace ? Oui, maman. Le livre est resté, Victorina. Oui, avec Nino. Le livre est resté. Ça sent le papier, un peu tiède. Et le carton, maman. Oui, dans l'air. Le livre reste sous la lampe. Un &lt;emphasis level="moderate"&gt;éclat de livre&lt;/emphasis&gt; tient sur le dos.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la lampe. Maman lisse un coin de page. Le livre a glissé, papa. Tu l'as vu, toi ? Oui, près de la table. On est bien, ici. Victorina tapote le dos du doigt. Il a une trace de doigt. Tu la vois, la trace ? Oui, maman. Le livre est resté, Victorina. Oui, avec Nino. Le livre est resté. Ça sent le papier, un peu tiède. Et le carton, maman. Oui, dans l'air. Le livre reste sous la lampe. Un &lt;emphasis&gt;éclat de livre&lt;/emphasis&gt; tient sur le dos.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2006,7 +2093,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2014,7 +2101,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2026,12 +2113,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2040,14 +2127,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de livre</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2059,11 +2150,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2072,27 +2163,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_dos; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit stop.
-enfant-m|Je me suis éloigné.
-enfant-m|Je suis allé vers maman.
-maman|Bravo.</t>
+          <t>narrateur|Ils restent près de la lampe.
+narrateur|Maman lisse un coin de page.
+enfant-f|Le livre a glissé, papa.
+papa|Tu l'as vu, toi ?
+enfant-f|Oui, près de la table.
+maman|On est bien, ici.
+narrateur|Victorina tapote le dos du doigt.
+enfant-f|Il a une trace de doigt.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le livre est resté, Victorina.
+enfant-f|Oui, avec Nino.
+copain|Le livre est resté.
+narrateur|Ça sent le papier, un peu tiède.
+enfant-f|Et le carton, maman.
+maman|Oui, dans l'air.
+narrateur|Le livre reste sous la lampe.
+narrateur|Un éclat de livre tient sur le dos.</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2170,6 +2279,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>